<commit_message>
Addressed category 2 issue
</commit_message>
<xml_diff>
--- a/backend/data/sample/VBAP_May2026.xlsx
+++ b/backend/data/sample/VBAP_May2026.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="149">
   <si>
     <t>MANDT</t>
   </si>
@@ -496,12 +496,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1344,8 +1347,8 @@
       <c r="CC2" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="CD2" s="1" t="s">
-        <v>103</v>
+      <c r="CD2" s="2">
+        <v>200.0</v>
       </c>
       <c r="CE2" s="1" t="s">
         <v>103</v>

</xml_diff>